<commit_message>
Add Gubbs ESD outlier detection for calibrators and unknowns. Updated the display tables for calibrators and unknowns.
</commit_message>
<xml_diff>
--- a/Change_Log.xlsx
+++ b/Change_Log.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roboy\iCloudDrive\Desktop\Python\Projects\4P_Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61260EAF-66D6-40DE-8473-84C4331F2C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4D4B77-9162-4A01-A393-6E11066DAFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-144" yWindow="876" windowWidth="17280" windowHeight="9960" xr2:uid="{C0F4DE78-8D30-4BD4-803A-299F828B33CD}"/>
+    <workbookView xWindow="1080" yWindow="276" windowWidth="13320" windowHeight="9960" xr2:uid="{C0F4DE78-8D30-4BD4-803A-299F828B33CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Update Ideas" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -70,6 +71,49 @@
   <si>
     <t>Update plotter.py with plot_residuals_vs_fitted function
 Update main_window to have a third tab "residuals vs fitted" with its own figure and canvas, and call the new function in open_csv</t>
+  </si>
+  <si>
+    <t>Better visualization of the LOQ range</t>
+  </si>
+  <si>
+    <t>It would look like a green shaded band between LLOQ and ULOQ on the calibration curve, giving the user an immediate visual sense of the reliable quantitation range.</t>
+  </si>
+  <si>
+    <t>Add lloq and uloq as parameters to plot_full_calibration and use ax.axvspan() to draw the shaded region</t>
+  </si>
+  <si>
+    <t>Turned the calibration and sample tables into tabs</t>
+  </si>
+  <si>
+    <t>Main update to main_window.py</t>
+  </si>
+  <si>
+    <t>Verification Package</t>
+  </si>
+  <si>
+    <t>Idea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Package for analyzing datasets for different types of analytical tests used to verify performance </t>
+  </si>
+  <si>
+    <t>Outlier test</t>
+  </si>
+  <si>
+    <t>Grubbs test for outliers</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>I implemented the Grubbs test for outlier detection in calibrator replicates. It calculates a G statistic for the most extreme value and compares it to a critical value based on sample size and significance level. I used the generalized ESD approach to detect multiple outliers iteratively. This is consistent with CLSI guidance for analytical method validation.</t>
+  </si>
+  <si>
+    <t>In-process</t>
+  </si>
+  <si>
+    <t>* helper_fnx.py - added grubbs and grubbs_esd functions
+*Created dictionary for listing outliers in the analysis script</t>
   </si>
 </sst>
 </file>
@@ -445,16 +489,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{198E4DBF-941C-4E7E-916A-9F1172FF2D6F}">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
     <col min="2" max="2" width="36.6640625" customWidth="1"/>
     <col min="3" max="3" width="44.33203125" customWidth="1"/>
     <col min="4" max="4" width="36.5546875" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -470,8 +515,11 @@
       <c r="E1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>46171</v>
       </c>
@@ -486,7 +534,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>46172</v>
       </c>
@@ -497,81 +545,115 @@
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>46172</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46173</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="144" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46173</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -747,5 +829,54 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5408C885-C812-4FA0-A954-770E05A76CC2}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46173</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>46173</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add PDF report generation with appendix
</commit_message>
<xml_diff>
--- a/Change_Log.xlsx
+++ b/Change_Log.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roboy\iCloudDrive\Desktop\Python\Projects\4P_Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4D4B77-9162-4A01-A393-6E11066DAFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44E33A4-9168-43C7-9205-E2CC155E3184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="276" windowWidth="13320" windowHeight="9960" xr2:uid="{C0F4DE78-8D30-4BD4-803A-299F828B33CD}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="20868" windowHeight="13296" xr2:uid="{C0F4DE78-8D30-4BD4-803A-299F828B33CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Update Ideas" sheetId="2" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -109,11 +110,48 @@
     <t>I implemented the Grubbs test for outlier detection in calibrator replicates. It calculates a G statistic for the most extreme value and compares it to a critical value based on sample size and significance level. I used the generalized ESD approach to detect multiple outliers iteratively. This is consistent with CLSI guidance for analytical method validation.</t>
   </si>
   <si>
+    <t xml:space="preserve">* helper_fnx.py - added grubbs and grubbs_esd functions
+*Created dictionary for listing outliers in the analysis script
+* Reporter - updated unknown_table and calibration_table functions to return a dictionary that includes a list of outliers, if any
+* Update main_window.py - updated init for table widget; updated call in open_csv function to include samlpe_outliers as an argument. </t>
+  </si>
+  <si>
+    <t>Linear/Log toggle of calibration curve</t>
+  </si>
+  <si>
+    <t>1. Add Qcheckbox to Pyside imports
+2. Add checkbox to the button row of init
+3. Add handler method
+4. Update plotter - modify plot_full_calibration function to accept log scale</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>General pattern for updating a GUI</t>
+  </si>
+  <si>
+    <t>Add widget --&gt; signal --&gt; connect signal to handler method --&gt; functional call</t>
+  </si>
+  <si>
+    <t>Generate a PDF report</t>
+  </si>
+  <si>
+    <t>Main report:
+1. Title and metadata
+2. Model parameters table
+3. Calibration curve plot
+4. Unknown samples summary table
+5. Calibrators summary table
+Appendix 6 - Unknown sample raw replicates
+Appendix 7 - Calibrator raw replicates
+Appendix 8 - Outlier flags</t>
+  </si>
+  <si>
     <t>In-process</t>
-  </si>
-  <si>
-    <t>* helper_fnx.py - added grubbs and grubbs_esd functions
-*Created dictionary for listing outliers in the analysis script</t>
   </si>
 </sst>
 </file>
@@ -495,7 +533,8 @@
     <col min="1" max="1" width="24.6640625" customWidth="1"/>
     <col min="2" max="2" width="36.6640625" customWidth="1"/>
     <col min="3" max="3" width="44.33203125" customWidth="1"/>
-    <col min="4" max="4" width="36.5546875" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" customWidth="1"/>
+    <col min="5" max="5" width="36.88671875" customWidth="1"/>
     <col min="6" max="6" width="31.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -581,7 +620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="144" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>46173</v>
       </c>
@@ -590,26 +629,44 @@
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="2"/>
+    <row r="7" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46176</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46176</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
@@ -879,4 +936,40 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60624C8D-6D4D-4671-BA33-A17F48BA2B25}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="34.88671875" customWidth="1"/>
+    <col min="3" max="3" width="54.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46176</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>